<commit_message>
Resolve I/O authority conflicts conservatively
</commit_message>
<xml_diff>
--- a/wiring/Mazak_Wiring_Master_7i97T_7i49_7i84U_Current_Authority.xlsx
+++ b/wiring/Mazak_Wiring_Master_7i97T_7i49_7i84U_Current_Authority.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2969" uniqueCount="475">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2969" uniqueCount="479">
   <si>
     <t>Mazak VQC-20/40 Wiring Master — Current Pin Authority</t>
   </si>
@@ -1255,181 +1255,193 @@
     <t>RLY-1 to SOL-13 Fujikoshi hydraulic valve</t>
   </si>
   <si>
+    <t>Conflict: connector_crossref.md identifies SOL-13 as gear-shift low; verify SOL-12/SOL-13 coil identity and high/low function before wiring</t>
+  </si>
+  <si>
+    <t>GEAR_LO_SOL</t>
+  </si>
+  <si>
+    <t>OUT8</t>
+  </si>
+  <si>
+    <t>gear-lo-sol</t>
+  </si>
+  <si>
+    <t>RLY-2 to SOL-12 Fujikoshi hydraulic valve</t>
+  </si>
+  <si>
+    <t>Conflict: connector_crossref.md omits SOL-12 and identifies SOL-13 as low; verify both gear-shift coils before wiring</t>
+  </si>
+  <si>
+    <t>TOOL_CLAMP_SOL</t>
+  </si>
+  <si>
+    <t>OUT9</t>
+  </si>
+  <si>
+    <t>tool-clamp-sol</t>
+  </si>
+  <si>
+    <t>RLY-3 to SOL-10 Fujikoshi hydraulic valve</t>
+  </si>
+  <si>
+    <t>Conflict: connector_crossref.md identifies SOL-10 as tool unclamp only; identify the clamp coil/valve before assigning OUT9</t>
+  </si>
+  <si>
+    <t>TOOL_UNCLAMP_SOL</t>
+  </si>
+  <si>
+    <t>OUT10</t>
+  </si>
+  <si>
+    <t>tool-unclamp-sol</t>
+  </si>
+  <si>
+    <t>RLY-4 to SOL-10 Fujikoshi hydraulic valve</t>
+  </si>
+  <si>
+    <t>Evidence supports SOL-10 tool unclamp; verify relay path and whether the valve is single-coil or dual-coil before energizing</t>
+  </si>
+  <si>
+    <t>COOLANT_ON</t>
+  </si>
+  <si>
+    <t>OUT11</t>
+  </si>
+  <si>
+    <t>flood-coolant</t>
+  </si>
+  <si>
+    <t>Coolant pump relay</t>
+  </si>
+  <si>
+    <t>May need interposing relay</t>
+  </si>
+  <si>
+    <t>LUBE_ON</t>
+  </si>
+  <si>
+    <t>OUT12</t>
+  </si>
+  <si>
+    <t>lube-on</t>
+  </si>
+  <si>
+    <t>Lube pump relay</t>
+  </si>
+  <si>
+    <t>ATC_FWD</t>
+  </si>
+  <si>
+    <t>ATC motor</t>
+  </si>
+  <si>
+    <t>OUT13</t>
+  </si>
+  <si>
+    <t>atc-fwd</t>
+  </si>
+  <si>
+    <t>ATC motor forward relay</t>
+  </si>
+  <si>
+    <t>Do not energize before interlocks are proven</t>
+  </si>
+  <si>
+    <t>ATC_REV</t>
+  </si>
+  <si>
+    <t>OUT14</t>
+  </si>
+  <si>
+    <t>atc-rev</t>
+  </si>
+  <si>
+    <t>ATC motor reverse relay</t>
+  </si>
+  <si>
+    <t>ALARM_OUT</t>
+  </si>
+  <si>
+    <t>OUT15</t>
+  </si>
+  <si>
+    <t>alarm-out</t>
+  </si>
+  <si>
+    <t>Alarm light or horn</t>
+  </si>
+  <si>
+    <t>HOLD_NOT_ORDERED</t>
+  </si>
+  <si>
+    <t>Confirm load and behavior</t>
+  </si>
+  <si>
+    <t>SECOND_SSERIAL_CARD</t>
+  </si>
+  <si>
+    <t>Expansion</t>
+  </si>
+  <si>
+    <t>REVIEW</t>
+  </si>
+  <si>
+    <t>Additional 7i84 or equivalent</t>
+  </si>
+  <si>
+    <t>phase2_conflict_review</t>
+  </si>
+  <si>
+    <t>Do not buy until final input count proves it is needed</t>
+  </si>
+  <si>
+    <t>Connector</t>
+  </si>
+  <si>
+    <t>Pin / Channel</t>
+  </si>
+  <si>
+    <t>Signal ID</t>
+  </si>
+  <si>
+    <t>HAL Net</t>
+  </si>
+  <si>
+    <t>Function / Load</t>
+  </si>
+  <si>
+    <t>Direction</t>
+  </si>
+  <si>
+    <t>Authority Status</t>
+  </si>
+  <si>
+    <t>Verification Notes</t>
+  </si>
+  <si>
+    <t>PLAN_VERIFY</t>
+  </si>
+  <si>
+    <t>Channel</t>
+  </si>
+  <si>
+    <t>Axis / Device</t>
+  </si>
+  <si>
+    <t>Source</t>
+  </si>
+  <si>
+    <t>Bit / Pin</t>
+  </si>
+  <si>
+    <t>Field Point / Load</t>
+  </si>
+  <si>
     <t>Measure coil voltage before selecting relay contacts</t>
   </si>
   <si>
-    <t>GEAR_LO_SOL</t>
-  </si>
-  <si>
-    <t>OUT8</t>
-  </si>
-  <si>
-    <t>gear-lo-sol</t>
-  </si>
-  <si>
-    <t>RLY-2 to SOL-12 Fujikoshi hydraulic valve</t>
-  </si>
-  <si>
-    <t>TOOL_CLAMP_SOL</t>
-  </si>
-  <si>
-    <t>OUT9</t>
-  </si>
-  <si>
-    <t>tool-clamp-sol</t>
-  </si>
-  <si>
-    <t>RLY-3 to SOL-10 Fujikoshi hydraulic valve</t>
-  </si>
-  <si>
     <t>Confirm single valve versus dual coil behavior</t>
-  </si>
-  <si>
-    <t>TOOL_UNCLAMP_SOL</t>
-  </si>
-  <si>
-    <t>OUT10</t>
-  </si>
-  <si>
-    <t>tool-unclamp-sol</t>
-  </si>
-  <si>
-    <t>RLY-4 to SOL-10 Fujikoshi hydraulic valve</t>
-  </si>
-  <si>
-    <t>COOLANT_ON</t>
-  </si>
-  <si>
-    <t>OUT11</t>
-  </si>
-  <si>
-    <t>flood-coolant</t>
-  </si>
-  <si>
-    <t>Coolant pump relay</t>
-  </si>
-  <si>
-    <t>May need interposing relay</t>
-  </si>
-  <si>
-    <t>LUBE_ON</t>
-  </si>
-  <si>
-    <t>OUT12</t>
-  </si>
-  <si>
-    <t>lube-on</t>
-  </si>
-  <si>
-    <t>Lube pump relay</t>
-  </si>
-  <si>
-    <t>ATC_FWD</t>
-  </si>
-  <si>
-    <t>ATC motor</t>
-  </si>
-  <si>
-    <t>OUT13</t>
-  </si>
-  <si>
-    <t>atc-fwd</t>
-  </si>
-  <si>
-    <t>ATC motor forward relay</t>
-  </si>
-  <si>
-    <t>Do not energize before interlocks are proven</t>
-  </si>
-  <si>
-    <t>ATC_REV</t>
-  </si>
-  <si>
-    <t>OUT14</t>
-  </si>
-  <si>
-    <t>atc-rev</t>
-  </si>
-  <si>
-    <t>ATC motor reverse relay</t>
-  </si>
-  <si>
-    <t>ALARM_OUT</t>
-  </si>
-  <si>
-    <t>OUT15</t>
-  </si>
-  <si>
-    <t>alarm-out</t>
-  </si>
-  <si>
-    <t>Alarm light or horn</t>
-  </si>
-  <si>
-    <t>HOLD_NOT_ORDERED</t>
-  </si>
-  <si>
-    <t>Confirm load and behavior</t>
-  </si>
-  <si>
-    <t>SECOND_SSERIAL_CARD</t>
-  </si>
-  <si>
-    <t>Expansion</t>
-  </si>
-  <si>
-    <t>REVIEW</t>
-  </si>
-  <si>
-    <t>Additional 7i84 or equivalent</t>
-  </si>
-  <si>
-    <t>phase2_conflict_review</t>
-  </si>
-  <si>
-    <t>Do not buy until final input count proves it is needed</t>
-  </si>
-  <si>
-    <t>Connector</t>
-  </si>
-  <si>
-    <t>Pin / Channel</t>
-  </si>
-  <si>
-    <t>Signal ID</t>
-  </si>
-  <si>
-    <t>HAL Net</t>
-  </si>
-  <si>
-    <t>Function / Load</t>
-  </si>
-  <si>
-    <t>Direction</t>
-  </si>
-  <si>
-    <t>Authority Status</t>
-  </si>
-  <si>
-    <t>Verification Notes</t>
-  </si>
-  <si>
-    <t>PLAN_VERIFY</t>
-  </si>
-  <si>
-    <t>Channel</t>
-  </si>
-  <si>
-    <t>Axis / Device</t>
-  </si>
-  <si>
-    <t>Source</t>
-  </si>
-  <si>
-    <t>Bit / Pin</t>
-  </si>
-  <si>
-    <t>Field Point / Load</t>
   </si>
   <si>
     <t>Subsystem</t>
@@ -4844,7 +4856,7 @@
         <v>409</v>
       </c>
       <c r="I82" s="5" t="s">
-        <v>40</v>
+        <v>103</v>
       </c>
       <c r="J82" s="4" t="s">
         <v>251</v>
@@ -4879,18 +4891,18 @@
         <v>414</v>
       </c>
       <c r="I83" s="5" t="s">
-        <v>40</v>
+        <v>103</v>
       </c>
       <c r="J83" s="4" t="s">
         <v>251</v>
       </c>
       <c r="K83" s="4" t="s">
-        <v>410</v>
+        <v>415</v>
       </c>
     </row>
     <row r="84" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A84" s="4" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="B84" s="4" t="s">
         <v>298</v>
@@ -4905,27 +4917,27 @@
         <v>55</v>
       </c>
       <c r="F84" s="4" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="G84" s="4" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="H84" s="4" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="I84" s="5" t="s">
-        <v>40</v>
+        <v>103</v>
       </c>
       <c r="J84" s="4" t="s">
         <v>251</v>
       </c>
       <c r="K84" s="4" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
     </row>
     <row r="85" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A85" s="4" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="B85" s="4" t="s">
         <v>298</v>
@@ -4940,13 +4952,13 @@
         <v>55</v>
       </c>
       <c r="F85" s="4" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="G85" s="4" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="H85" s="4" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="I85" s="5" t="s">
         <v>40</v>
@@ -4955,12 +4967,12 @@
         <v>251</v>
       </c>
       <c r="K85" s="4" t="s">
-        <v>419</v>
+        <v>425</v>
       </c>
     </row>
     <row r="86" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A86" s="4" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="B86" s="4" t="s">
         <v>212</v>
@@ -4975,13 +4987,13 @@
         <v>55</v>
       </c>
       <c r="F86" s="4" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="G86" s="4" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="H86" s="4" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="I86" s="5" t="s">
         <v>40</v>
@@ -4990,12 +5002,12 @@
         <v>66</v>
       </c>
       <c r="K86" s="4" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
     </row>
     <row r="87" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A87" s="4" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="B87" s="4" t="s">
         <v>345</v>
@@ -5010,13 +5022,13 @@
         <v>55</v>
       </c>
       <c r="F87" s="4" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="G87" s="4" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="H87" s="4" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="I87" s="5" t="s">
         <v>40</v>
@@ -5025,15 +5037,15 @@
         <v>66</v>
       </c>
       <c r="K87" s="4" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
     </row>
     <row r="88" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A88" s="4" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="B88" s="4" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="C88" s="4" t="s">
         <v>69</v>
@@ -5045,13 +5057,13 @@
         <v>55</v>
       </c>
       <c r="F88" s="4" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="G88" s="4" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="H88" s="4" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="I88" s="5" t="s">
         <v>40</v>
@@ -5060,15 +5072,15 @@
         <v>66</v>
       </c>
       <c r="K88" s="4" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
     </row>
     <row r="89" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A89" s="4" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="B89" s="4" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="C89" s="4" t="s">
         <v>69</v>
@@ -5080,13 +5092,13 @@
         <v>55</v>
       </c>
       <c r="F89" s="4" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="G89" s="4" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="H89" s="4" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="I89" s="5" t="s">
         <v>365</v>
@@ -5095,12 +5107,12 @@
         <v>66</v>
       </c>
       <c r="K89" s="4" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
     </row>
     <row r="90" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A90" s="4" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="B90" s="4" t="s">
         <v>361</v>
@@ -5115,33 +5127,33 @@
         <v>55</v>
       </c>
       <c r="F90" s="4" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="G90" s="4" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="H90" s="4" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="I90" s="5" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="J90" s="4" t="s">
         <v>66</v>
       </c>
       <c r="K90" s="4" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
     </row>
     <row r="91" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A91" s="4" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="B91" s="4" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="C91" s="4" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="D91" s="4" t="s">
         <v>63</v>
@@ -5156,16 +5168,16 @@
         <v>63</v>
       </c>
       <c r="H91" s="4" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="I91" s="7" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="J91" s="4" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="K91" s="4" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
     </row>
   </sheetData>
@@ -5199,28 +5211,28 @@
   <sheetData>
     <row r="1" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>457</v>
+        <v>459</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
@@ -5295,7 +5307,7 @@
         <v>69</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="H4" s="4" t="s">
         <v>74</v>
@@ -5321,7 +5333,7 @@
         <v>76</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="H5" s="4" t="s">
         <v>80</v>
@@ -5347,7 +5359,7 @@
         <v>69</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="H6" s="4" t="s">
         <v>74</v>
@@ -5373,7 +5385,7 @@
         <v>76</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="H7" s="4" t="s">
         <v>89</v>
@@ -5399,7 +5411,7 @@
         <v>69</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="H8" s="4" t="s">
         <v>74</v>
@@ -5425,7 +5437,7 @@
         <v>76</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="H9" s="4" t="s">
         <v>98</v>
@@ -5477,7 +5489,7 @@
         <v>76</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="H11" s="4" t="s">
         <v>109</v>
@@ -5971,7 +5983,7 @@
         <v>192</v>
       </c>
       <c r="G30" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="H30" s="4" t="s">
         <v>195</v>
@@ -5997,7 +6009,7 @@
         <v>192</v>
       </c>
       <c r="G31" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="H31" s="4" t="s">
         <v>199</v>
@@ -6023,7 +6035,7 @@
         <v>69</v>
       </c>
       <c r="G32" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="H32" s="4" t="s">
         <v>206</v>
@@ -6049,7 +6061,7 @@
         <v>69</v>
       </c>
       <c r="G33" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="H33" s="4" t="s">
         <v>206</v>
@@ -6075,7 +6087,7 @@
         <v>69</v>
       </c>
       <c r="G34" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="H34" s="4" t="s">
         <v>206</v>
@@ -6189,25 +6201,25 @@
   <sheetData>
     <row r="1" ht="32" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>457</v>
+        <v>459</v>
       </c>
       <c r="B1" s="3" t="s">
+        <v>466</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>467</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>460</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>468</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>463</v>
+      </c>
+      <c r="G1" s="3" t="s">
         <v>464</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>465</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>458</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>466</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>461</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>462</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -6227,7 +6239,7 @@
         <v>41</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="G2" s="4" t="s">
         <v>42</v>
@@ -6250,7 +6262,7 @@
         <v>41</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="G3" s="4" t="s">
         <v>42</v>
@@ -6273,7 +6285,7 @@
         <v>41</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="G4" s="4" t="s">
         <v>42</v>
@@ -6308,28 +6320,28 @@
   <sheetData>
     <row r="1" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
+        <v>462</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>457</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>469</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>459</v>
+      </c>
+      <c r="E1" s="3" t="s">
         <v>460</v>
       </c>
-      <c r="B1" s="3" t="s">
-        <v>455</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>467</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>457</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>458</v>
-      </c>
       <c r="F1" s="3" t="s">
-        <v>468</v>
+        <v>470</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
@@ -6352,7 +6364,7 @@
         <v>230</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="H2" s="4" t="s">
         <v>231</v>
@@ -6378,7 +6390,7 @@
         <v>234</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="H3" s="4" t="s">
         <v>235</v>
@@ -6404,7 +6416,7 @@
         <v>240</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="H4" s="4" t="s">
         <v>241</v>
@@ -6430,7 +6442,7 @@
         <v>245</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="H5" s="4" t="s">
         <v>246</v>
@@ -6456,7 +6468,7 @@
         <v>250</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="H6" s="4" t="s">
         <v>252</v>
@@ -6482,7 +6494,7 @@
         <v>256</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="H7" s="4" t="s">
         <v>252</v>
@@ -6664,7 +6676,7 @@
         <v>275</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="H14" s="4" t="s">
         <v>276</v>
@@ -6690,7 +6702,7 @@
         <v>280</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="H15" s="4" t="s">
         <v>281</v>
@@ -6716,7 +6728,7 @@
         <v>285</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="H16" s="4" t="s">
         <v>286</v>
@@ -6742,7 +6754,7 @@
         <v>291</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="H17" s="4" t="s">
         <v>292</v>
@@ -6768,7 +6780,7 @@
         <v>296</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="H18" s="4" t="s">
         <v>292</v>
@@ -6794,7 +6806,7 @@
         <v>301</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="H19" s="4" t="s">
         <v>302</v>
@@ -6820,7 +6832,7 @@
         <v>306</v>
       </c>
       <c r="G20" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="H20" s="4" t="s">
         <v>307</v>
@@ -6846,7 +6858,7 @@
         <v>312</v>
       </c>
       <c r="G21" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="H21" s="4" t="s">
         <v>252</v>
@@ -6872,7 +6884,7 @@
         <v>316</v>
       </c>
       <c r="G22" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="H22" s="4" t="s">
         <v>252</v>
@@ -6898,7 +6910,7 @@
         <v>321</v>
       </c>
       <c r="G23" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="H23" s="4" t="s">
         <v>322</v>
@@ -6924,7 +6936,7 @@
         <v>326</v>
       </c>
       <c r="G24" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="H24" s="4" t="s">
         <v>322</v>
@@ -6950,7 +6962,7 @@
         <v>330</v>
       </c>
       <c r="G25" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="H25" s="4" t="s">
         <v>322</v>
@@ -6976,7 +6988,7 @@
         <v>334</v>
       </c>
       <c r="G26" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="H26" s="4" t="s">
         <v>322</v>
@@ -7002,7 +7014,7 @@
         <v>338</v>
       </c>
       <c r="G27" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="H27" s="4" t="s">
         <v>322</v>
@@ -7028,7 +7040,7 @@
         <v>342</v>
       </c>
       <c r="G28" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="H28" s="4" t="s">
         <v>343</v>
@@ -7054,7 +7066,7 @@
         <v>348</v>
       </c>
       <c r="G29" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="H29" s="4" t="s">
         <v>349</v>
@@ -7080,7 +7092,7 @@
         <v>353</v>
       </c>
       <c r="G30" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="H30" s="4" t="s">
         <v>349</v>
@@ -7106,7 +7118,7 @@
         <v>358</v>
       </c>
       <c r="G31" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="H31" s="4" t="s">
         <v>359</v>
@@ -7210,7 +7222,7 @@
         <v>378</v>
       </c>
       <c r="G35" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="H35" s="4" t="s">
         <v>379</v>
@@ -7236,7 +7248,7 @@
         <v>383</v>
       </c>
       <c r="G36" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="H36" s="4" t="s">
         <v>384</v>
@@ -7262,7 +7274,7 @@
         <v>388</v>
       </c>
       <c r="G37" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="H37" s="4" t="s">
         <v>384</v>
@@ -7288,7 +7300,7 @@
         <v>392</v>
       </c>
       <c r="G38" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="H38" s="4" t="s">
         <v>384</v>
@@ -7392,7 +7404,7 @@
         <v>404</v>
       </c>
       <c r="G42" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="H42" s="4" t="s">
         <v>405</v>
@@ -7418,10 +7430,10 @@
         <v>409</v>
       </c>
       <c r="G43" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="H43" s="4" t="s">
-        <v>410</v>
+        <v>471</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.25">
@@ -7444,10 +7456,10 @@
         <v>414</v>
       </c>
       <c r="G44" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="H44" s="4" t="s">
-        <v>410</v>
+        <v>471</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.25">
@@ -7458,22 +7470,22 @@
         <v>55</v>
       </c>
       <c r="C45" s="4" t="s">
+        <v>417</v>
+      </c>
+      <c r="D45" s="4" t="s">
         <v>416</v>
       </c>
-      <c r="D45" s="4" t="s">
-        <v>415</v>
-      </c>
       <c r="E45" s="4" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="F45" s="4" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="G45" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="H45" s="4" t="s">
-        <v>419</v>
+        <v>472</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.25">
@@ -7484,22 +7496,22 @@
         <v>55</v>
       </c>
       <c r="C46" s="4" t="s">
+        <v>422</v>
+      </c>
+      <c r="D46" s="4" t="s">
         <v>421</v>
       </c>
-      <c r="D46" s="4" t="s">
-        <v>420</v>
-      </c>
       <c r="E46" s="4" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="F46" s="4" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="G46" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="H46" s="4" t="s">
-        <v>419</v>
+        <v>472</v>
       </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.25">
@@ -7510,22 +7522,22 @@
         <v>55</v>
       </c>
       <c r="C47" s="4" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="D47" s="4" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="E47" s="4" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="F47" s="4" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="G47" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="H47" s="4" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.25">
@@ -7536,22 +7548,22 @@
         <v>55</v>
       </c>
       <c r="C48" s="4" t="s">
+        <v>432</v>
+      </c>
+      <c r="D48" s="4" t="s">
+        <v>431</v>
+      </c>
+      <c r="E48" s="4" t="s">
+        <v>433</v>
+      </c>
+      <c r="F48" s="4" t="s">
+        <v>434</v>
+      </c>
+      <c r="G48" s="4" t="s">
+        <v>465</v>
+      </c>
+      <c r="H48" s="4" t="s">
         <v>430</v>
-      </c>
-      <c r="D48" s="4" t="s">
-        <v>429</v>
-      </c>
-      <c r="E48" s="4" t="s">
-        <v>431</v>
-      </c>
-      <c r="F48" s="4" t="s">
-        <v>432</v>
-      </c>
-      <c r="G48" s="4" t="s">
-        <v>463</v>
-      </c>
-      <c r="H48" s="4" t="s">
-        <v>428</v>
       </c>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.25">
@@ -7562,22 +7574,22 @@
         <v>55</v>
       </c>
       <c r="C49" s="4" t="s">
+        <v>437</v>
+      </c>
+      <c r="D49" s="4" t="s">
         <v>435</v>
       </c>
-      <c r="D49" s="4" t="s">
-        <v>433</v>
-      </c>
       <c r="E49" s="4" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="F49" s="4" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="G49" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="H49" s="4" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.25">
@@ -7588,22 +7600,22 @@
         <v>55</v>
       </c>
       <c r="C50" s="4" t="s">
+        <v>442</v>
+      </c>
+      <c r="D50" s="4" t="s">
+        <v>441</v>
+      </c>
+      <c r="E50" s="4" t="s">
+        <v>443</v>
+      </c>
+      <c r="F50" s="4" t="s">
+        <v>444</v>
+      </c>
+      <c r="G50" s="4" t="s">
+        <v>465</v>
+      </c>
+      <c r="H50" s="4" t="s">
         <v>440</v>
-      </c>
-      <c r="D50" s="4" t="s">
-        <v>439</v>
-      </c>
-      <c r="E50" s="4" t="s">
-        <v>441</v>
-      </c>
-      <c r="F50" s="4" t="s">
-        <v>442</v>
-      </c>
-      <c r="G50" s="4" t="s">
-        <v>463</v>
-      </c>
-      <c r="H50" s="4" t="s">
-        <v>438</v>
       </c>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.25">
@@ -7614,22 +7626,22 @@
         <v>55</v>
       </c>
       <c r="C51" s="4" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="D51" s="4" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="E51" s="4" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="F51" s="4" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="G51" s="4" t="s">
         <v>365</v>
       </c>
       <c r="H51" s="4" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
     </row>
   </sheetData>
@@ -7662,31 +7674,31 @@
   <sheetData>
     <row r="1" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
+        <v>460</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>459</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>473</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>462</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>474</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>457</v>
+      </c>
+      <c r="G1" s="3" t="s">
         <v>458</v>
       </c>
-      <c r="B1" s="3" t="s">
-        <v>457</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>469</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>460</v>
-      </c>
-      <c r="E1" s="3" t="s">
+      <c r="H1" s="3" t="s">
+        <v>463</v>
+      </c>
+      <c r="I1" s="3" t="s">
         <v>470</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>455</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>456</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>461</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>468</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
@@ -7712,7 +7724,7 @@
         <v>37</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I2" s="4" t="s">
         <v>39</v>
@@ -7741,7 +7753,7 @@
         <v>44</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I3" s="4" t="s">
         <v>46</v>
@@ -7770,7 +7782,7 @@
         <v>48</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I4" s="4" t="s">
         <v>50</v>
@@ -7828,7 +7840,7 @@
         <v>71</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I6" s="4" t="s">
         <v>73</v>
@@ -7857,7 +7869,7 @@
         <v>77</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I7" s="4" t="s">
         <v>79</v>
@@ -7886,7 +7898,7 @@
         <v>82</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I8" s="4" t="s">
         <v>84</v>
@@ -7915,7 +7927,7 @@
         <v>86</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I9" s="4" t="s">
         <v>88</v>
@@ -7944,7 +7956,7 @@
         <v>91</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I10" s="4" t="s">
         <v>93</v>
@@ -7973,7 +7985,7 @@
         <v>95</v>
       </c>
       <c r="H11" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I11" s="4" t="s">
         <v>97</v>
@@ -8031,7 +8043,7 @@
         <v>106</v>
       </c>
       <c r="H13" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I13" s="4" t="s">
         <v>108</v>
@@ -8350,7 +8362,7 @@
         <v>203</v>
       </c>
       <c r="H24" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I24" s="4" t="s">
         <v>205</v>
@@ -8379,7 +8391,7 @@
         <v>208</v>
       </c>
       <c r="H25" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I25" s="4" t="s">
         <v>210</v>
@@ -8408,7 +8420,7 @@
         <v>213</v>
       </c>
       <c r="H26" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I26" s="4" t="s">
         <v>215</v>
@@ -8437,7 +8449,7 @@
         <v>238</v>
       </c>
       <c r="H27" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I27" s="4" t="s">
         <v>240</v>
@@ -8466,7 +8478,7 @@
         <v>243</v>
       </c>
       <c r="H28" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I28" s="4" t="s">
         <v>245</v>
@@ -8495,7 +8507,7 @@
         <v>248</v>
       </c>
       <c r="H29" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I29" s="4" t="s">
         <v>250</v>
@@ -8524,7 +8536,7 @@
         <v>254</v>
       </c>
       <c r="H30" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I30" s="4" t="s">
         <v>256</v>
@@ -8553,7 +8565,7 @@
         <v>273</v>
       </c>
       <c r="H31" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I31" s="4" t="s">
         <v>275</v>
@@ -8582,7 +8594,7 @@
         <v>278</v>
       </c>
       <c r="H32" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I32" s="4" t="s">
         <v>280</v>
@@ -8611,7 +8623,7 @@
         <v>283</v>
       </c>
       <c r="H33" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I33" s="4" t="s">
         <v>285</v>
@@ -8640,7 +8652,7 @@
         <v>289</v>
       </c>
       <c r="H34" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I34" s="4" t="s">
         <v>291</v>
@@ -8669,7 +8681,7 @@
         <v>294</v>
       </c>
       <c r="H35" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I35" s="4" t="s">
         <v>296</v>
@@ -8698,7 +8710,7 @@
         <v>299</v>
       </c>
       <c r="H36" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I36" s="4" t="s">
         <v>301</v>
@@ -8727,7 +8739,7 @@
         <v>304</v>
       </c>
       <c r="H37" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I37" s="4" t="s">
         <v>306</v>
@@ -8756,7 +8768,7 @@
         <v>310</v>
       </c>
       <c r="H38" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I38" s="4" t="s">
         <v>312</v>
@@ -8785,7 +8797,7 @@
         <v>314</v>
       </c>
       <c r="H39" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I39" s="4" t="s">
         <v>316</v>
@@ -8814,7 +8826,7 @@
         <v>319</v>
       </c>
       <c r="H40" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I40" s="4" t="s">
         <v>321</v>
@@ -8843,7 +8855,7 @@
         <v>324</v>
       </c>
       <c r="H41" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I41" s="4" t="s">
         <v>326</v>
@@ -8872,7 +8884,7 @@
         <v>328</v>
       </c>
       <c r="H42" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I42" s="4" t="s">
         <v>330</v>
@@ -8901,7 +8913,7 @@
         <v>332</v>
       </c>
       <c r="H43" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I43" s="4" t="s">
         <v>334</v>
@@ -8930,7 +8942,7 @@
         <v>336</v>
       </c>
       <c r="H44" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I44" s="4" t="s">
         <v>338</v>
@@ -8959,7 +8971,7 @@
         <v>340</v>
       </c>
       <c r="H45" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I45" s="4" t="s">
         <v>342</v>
@@ -8988,7 +9000,7 @@
         <v>346</v>
       </c>
       <c r="H46" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I46" s="4" t="s">
         <v>348</v>
@@ -9017,7 +9029,7 @@
         <v>351</v>
       </c>
       <c r="H47" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I47" s="4" t="s">
         <v>353</v>
@@ -9046,7 +9058,7 @@
         <v>356</v>
       </c>
       <c r="H48" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I48" s="4" t="s">
         <v>358</v>
@@ -9162,7 +9174,7 @@
         <v>376</v>
       </c>
       <c r="H52" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I52" s="4" t="s">
         <v>378</v>
@@ -9191,7 +9203,7 @@
         <v>381</v>
       </c>
       <c r="H53" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I53" s="4" t="s">
         <v>383</v>
@@ -9220,7 +9232,7 @@
         <v>386</v>
       </c>
       <c r="H54" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I54" s="4" t="s">
         <v>388</v>
@@ -9249,7 +9261,7 @@
         <v>390</v>
       </c>
       <c r="H55" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I55" s="4" t="s">
         <v>392</v>
@@ -9278,7 +9290,7 @@
         <v>402</v>
       </c>
       <c r="H56" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I56" s="4" t="s">
         <v>404</v>
@@ -9307,7 +9319,7 @@
         <v>407</v>
       </c>
       <c r="H57" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I57" s="4" t="s">
         <v>409</v>
@@ -9336,7 +9348,7 @@
         <v>412</v>
       </c>
       <c r="H58" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I58" s="4" t="s">
         <v>414</v>
@@ -9344,10 +9356,10 @@
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A59" s="4" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="B59" s="4" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="C59" s="4" t="s">
         <v>298</v>
@@ -9362,21 +9374,21 @@
         <v>55</v>
       </c>
       <c r="G59" s="4" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="H59" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I59" s="4" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A60" s="4" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="B60" s="4" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="C60" s="4" t="s">
         <v>298</v>
@@ -9391,21 +9403,21 @@
         <v>55</v>
       </c>
       <c r="G60" s="4" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="H60" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I60" s="4" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A61" s="4" t="s">
+        <v>428</v>
+      </c>
+      <c r="B61" s="4" t="s">
         <v>426</v>
-      </c>
-      <c r="B61" s="4" t="s">
-        <v>424</v>
       </c>
       <c r="C61" s="4" t="s">
         <v>212</v>
@@ -9420,21 +9432,21 @@
         <v>55</v>
       </c>
       <c r="G61" s="4" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="H61" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I61" s="4" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A62" s="4" t="s">
+        <v>433</v>
+      </c>
+      <c r="B62" s="4" t="s">
         <v>431</v>
-      </c>
-      <c r="B62" s="4" t="s">
-        <v>429</v>
       </c>
       <c r="C62" s="4" t="s">
         <v>345</v>
@@ -9449,24 +9461,24 @@
         <v>55</v>
       </c>
       <c r="G62" s="4" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="H62" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I62" s="4" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A63" s="4" t="s">
+        <v>438</v>
+      </c>
+      <c r="B63" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="C63" s="4" t="s">
         <v>436</v>
-      </c>
-      <c r="B63" s="4" t="s">
-        <v>433</v>
-      </c>
-      <c r="C63" s="4" t="s">
-        <v>434</v>
       </c>
       <c r="D63" s="4" t="s">
         <v>69</v>
@@ -9478,24 +9490,24 @@
         <v>55</v>
       </c>
       <c r="G63" s="4" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="H63" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I63" s="4" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A64" s="4" t="s">
+        <v>443</v>
+      </c>
+      <c r="B64" s="4" t="s">
         <v>441</v>
       </c>
-      <c r="B64" s="4" t="s">
-        <v>439</v>
-      </c>
       <c r="C64" s="4" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="D64" s="4" t="s">
         <v>69</v>
@@ -9507,21 +9519,21 @@
         <v>55</v>
       </c>
       <c r="G64" s="4" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="H64" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I64" s="4" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A65" s="4" t="s">
+        <v>447</v>
+      </c>
+      <c r="B65" s="4" t="s">
         <v>445</v>
-      </c>
-      <c r="B65" s="4" t="s">
-        <v>443</v>
       </c>
       <c r="C65" s="4" t="s">
         <v>361</v>
@@ -9536,13 +9548,13 @@
         <v>55</v>
       </c>
       <c r="G65" s="4" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="H65" s="4" t="s">
         <v>365</v>
       </c>
       <c r="I65" s="4" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
     </row>
   </sheetData>
@@ -9576,36 +9588,36 @@
   <sheetData>
     <row r="1" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>471</v>
+        <v>475</v>
       </c>
       <c r="B1" s="3" t="s">
+        <v>459</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>473</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>474</v>
+      </c>
+      <c r="E1" s="3" t="s">
         <v>457</v>
       </c>
-      <c r="C1" s="3" t="s">
-        <v>469</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>470</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>455</v>
-      </c>
       <c r="F1" s="3" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>472</v>
+        <v>476</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>32</v>
@@ -9626,7 +9638,7 @@
         <v>38</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I2" s="4" t="s">
         <v>42</v>
@@ -9634,7 +9646,7 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>43</v>
@@ -9655,7 +9667,7 @@
         <v>45</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I3" s="4" t="s">
         <v>42</v>
@@ -9663,7 +9675,7 @@
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>47</v>
@@ -9684,7 +9696,7 @@
         <v>49</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I4" s="4" t="s">
         <v>42</v>
@@ -9692,7 +9704,7 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="B5" s="4" t="s">
         <v>51</v>
@@ -9721,7 +9733,7 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>68</v>
@@ -9742,7 +9754,7 @@
         <v>72</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I6" s="4" t="s">
         <v>74</v>
@@ -9750,7 +9762,7 @@
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="B7" s="4" t="s">
         <v>75</v>
@@ -9771,7 +9783,7 @@
         <v>78</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I7" s="4" t="s">
         <v>80</v>
@@ -9779,7 +9791,7 @@
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="B8" s="4" t="s">
         <v>81</v>
@@ -9800,7 +9812,7 @@
         <v>83</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I8" s="4" t="s">
         <v>74</v>
@@ -9808,7 +9820,7 @@
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="B9" s="4" t="s">
         <v>85</v>
@@ -9829,7 +9841,7 @@
         <v>87</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I9" s="4" t="s">
         <v>89</v>
@@ -9837,7 +9849,7 @@
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="B10" s="4" t="s">
         <v>90</v>
@@ -9858,7 +9870,7 @@
         <v>92</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I10" s="4" t="s">
         <v>74</v>
@@ -9866,7 +9878,7 @@
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="B11" s="4" t="s">
         <v>94</v>
@@ -9887,7 +9899,7 @@
         <v>96</v>
       </c>
       <c r="H11" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I11" s="4" t="s">
         <v>98</v>
@@ -9895,7 +9907,7 @@
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
-        <v>474</v>
+        <v>478</v>
       </c>
       <c r="B12" s="4" t="s">
         <v>99</v>
@@ -9924,7 +9936,7 @@
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="B13" s="4" t="s">
         <v>105</v>
@@ -9945,7 +9957,7 @@
         <v>107</v>
       </c>
       <c r="H13" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I13" s="4" t="s">
         <v>109</v>
@@ -9953,7 +9965,7 @@
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="B14" s="4" t="s">
         <v>143</v>
@@ -9982,7 +9994,7 @@
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="B15" s="4" t="s">
         <v>152</v>
@@ -10011,7 +10023,7 @@
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="B16" s="4" t="s">
         <v>156</v>
@@ -10040,7 +10052,7 @@
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="B17" s="4" t="s">
         <v>160</v>
@@ -10069,7 +10081,7 @@
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="B18" s="4" t="s">
         <v>164</v>
@@ -10098,7 +10110,7 @@
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="B19" s="4" t="s">
         <v>168</v>
@@ -10127,7 +10139,7 @@
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="B20" s="4" t="s">
         <v>172</v>
@@ -10156,7 +10168,7 @@
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="B21" s="4" t="s">
         <v>176</v>
@@ -10185,7 +10197,7 @@
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="B22" s="4" t="s">
         <v>180</v>
@@ -10214,7 +10226,7 @@
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="B23" s="4" t="s">
         <v>184</v>
@@ -10243,7 +10255,7 @@
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="B24" s="4" t="s">
         <v>190</v>
@@ -10264,7 +10276,7 @@
         <v>63</v>
       </c>
       <c r="H24" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I24" s="4" t="s">
         <v>195</v>
@@ -10272,7 +10284,7 @@
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="B25" s="4" t="s">
         <v>196</v>
@@ -10293,7 +10305,7 @@
         <v>63</v>
       </c>
       <c r="H25" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I25" s="4" t="s">
         <v>199</v>
@@ -10301,7 +10313,7 @@
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="B26" s="4" t="s">
         <v>200</v>
@@ -10322,7 +10334,7 @@
         <v>204</v>
       </c>
       <c r="H26" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I26" s="4" t="s">
         <v>206</v>
@@ -10330,7 +10342,7 @@
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" s="5" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="B27" s="4" t="s">
         <v>207</v>
@@ -10351,7 +10363,7 @@
         <v>209</v>
       </c>
       <c r="H27" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I27" s="4" t="s">
         <v>206</v>
@@ -10359,7 +10371,7 @@
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" s="5" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="B28" s="4" t="s">
         <v>211</v>
@@ -10380,7 +10392,7 @@
         <v>214</v>
       </c>
       <c r="H28" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I28" s="4" t="s">
         <v>206</v>
@@ -10388,7 +10400,7 @@
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" s="5" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="B29" s="4" t="s">
         <v>226</v>
@@ -10409,7 +10421,7 @@
         <v>63</v>
       </c>
       <c r="H29" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I29" s="4" t="s">
         <v>231</v>
@@ -10417,7 +10429,7 @@
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" s="5" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="B30" s="4" t="s">
         <v>232</v>
@@ -10438,7 +10450,7 @@
         <v>63</v>
       </c>
       <c r="H30" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I30" s="4" t="s">
         <v>235</v>
@@ -10446,7 +10458,7 @@
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" s="5" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="B31" s="4" t="s">
         <v>236</v>
@@ -10467,7 +10479,7 @@
         <v>239</v>
       </c>
       <c r="H31" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I31" s="4" t="s">
         <v>241</v>
@@ -10475,7 +10487,7 @@
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" s="5" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="B32" s="4" t="s">
         <v>242</v>
@@ -10496,7 +10508,7 @@
         <v>244</v>
       </c>
       <c r="H32" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I32" s="4" t="s">
         <v>246</v>
@@ -10504,7 +10516,7 @@
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" s="5" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="B33" s="4" t="s">
         <v>247</v>
@@ -10525,7 +10537,7 @@
         <v>249</v>
       </c>
       <c r="H33" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I33" s="4" t="s">
         <v>252</v>
@@ -10533,7 +10545,7 @@
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" s="5" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="B34" s="4" t="s">
         <v>253</v>
@@ -10554,7 +10566,7 @@
         <v>255</v>
       </c>
       <c r="H34" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I34" s="4" t="s">
         <v>252</v>
@@ -10562,7 +10574,7 @@
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" s="5" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="B35" s="4" t="s">
         <v>271</v>
@@ -10583,7 +10595,7 @@
         <v>274</v>
       </c>
       <c r="H35" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I35" s="4" t="s">
         <v>276</v>
@@ -10591,7 +10603,7 @@
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" s="5" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="B36" s="4" t="s">
         <v>277</v>
@@ -10612,7 +10624,7 @@
         <v>279</v>
       </c>
       <c r="H36" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I36" s="4" t="s">
         <v>281</v>
@@ -10620,7 +10632,7 @@
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" s="5" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="B37" s="4" t="s">
         <v>282</v>
@@ -10641,7 +10653,7 @@
         <v>284</v>
       </c>
       <c r="H37" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I37" s="4" t="s">
         <v>286</v>
@@ -10649,7 +10661,7 @@
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" s="5" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="B38" s="4" t="s">
         <v>287</v>
@@ -10670,7 +10682,7 @@
         <v>290</v>
       </c>
       <c r="H38" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I38" s="4" t="s">
         <v>292</v>
@@ -10678,7 +10690,7 @@
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" s="5" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="B39" s="4" t="s">
         <v>293</v>
@@ -10699,7 +10711,7 @@
         <v>295</v>
       </c>
       <c r="H39" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I39" s="4" t="s">
         <v>292</v>
@@ -10707,7 +10719,7 @@
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" s="5" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="B40" s="4" t="s">
         <v>297</v>
@@ -10728,7 +10740,7 @@
         <v>300</v>
       </c>
       <c r="H40" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I40" s="4" t="s">
         <v>302</v>
@@ -10736,7 +10748,7 @@
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" s="5" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="B41" s="4" t="s">
         <v>303</v>
@@ -10757,7 +10769,7 @@
         <v>305</v>
       </c>
       <c r="H41" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I41" s="4" t="s">
         <v>307</v>
@@ -10765,7 +10777,7 @@
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" s="5" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="B42" s="4" t="s">
         <v>308</v>
@@ -10786,7 +10798,7 @@
         <v>311</v>
       </c>
       <c r="H42" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I42" s="4" t="s">
         <v>252</v>
@@ -10794,7 +10806,7 @@
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" s="5" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="B43" s="4" t="s">
         <v>313</v>
@@ -10815,7 +10827,7 @@
         <v>315</v>
       </c>
       <c r="H43" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I43" s="4" t="s">
         <v>252</v>
@@ -10823,7 +10835,7 @@
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" s="5" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="B44" s="4" t="s">
         <v>317</v>
@@ -10844,7 +10856,7 @@
         <v>320</v>
       </c>
       <c r="H44" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I44" s="4" t="s">
         <v>322</v>
@@ -10852,7 +10864,7 @@
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" s="5" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="B45" s="4" t="s">
         <v>323</v>
@@ -10873,7 +10885,7 @@
         <v>325</v>
       </c>
       <c r="H45" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I45" s="4" t="s">
         <v>322</v>
@@ -10881,7 +10893,7 @@
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46" s="5" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="B46" s="4" t="s">
         <v>327</v>
@@ -10902,7 +10914,7 @@
         <v>329</v>
       </c>
       <c r="H46" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I46" s="4" t="s">
         <v>322</v>
@@ -10910,7 +10922,7 @@
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47" s="5" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="B47" s="4" t="s">
         <v>331</v>
@@ -10931,7 +10943,7 @@
         <v>333</v>
       </c>
       <c r="H47" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I47" s="4" t="s">
         <v>322</v>
@@ -10939,7 +10951,7 @@
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" s="5" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="B48" s="4" t="s">
         <v>335</v>
@@ -10960,7 +10972,7 @@
         <v>337</v>
       </c>
       <c r="H48" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I48" s="4" t="s">
         <v>322</v>
@@ -10968,7 +10980,7 @@
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A49" s="5" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="B49" s="4" t="s">
         <v>339</v>
@@ -10989,7 +11001,7 @@
         <v>341</v>
       </c>
       <c r="H49" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I49" s="4" t="s">
         <v>343</v>
@@ -10997,7 +11009,7 @@
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A50" s="5" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="B50" s="4" t="s">
         <v>344</v>
@@ -11018,7 +11030,7 @@
         <v>347</v>
       </c>
       <c r="H50" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I50" s="4" t="s">
         <v>349</v>
@@ -11026,7 +11038,7 @@
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A51" s="5" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="B51" s="4" t="s">
         <v>350</v>
@@ -11047,7 +11059,7 @@
         <v>352</v>
       </c>
       <c r="H51" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I51" s="4" t="s">
         <v>349</v>
@@ -11055,7 +11067,7 @@
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A52" s="5" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="B52" s="4" t="s">
         <v>354</v>
@@ -11076,7 +11088,7 @@
         <v>357</v>
       </c>
       <c r="H52" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I52" s="4" t="s">
         <v>359</v>
@@ -11084,7 +11096,7 @@
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A53" s="5" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="B53" s="4" t="s">
         <v>360</v>
@@ -11113,7 +11125,7 @@
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A54" s="5" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="B54" s="4" t="s">
         <v>367</v>
@@ -11142,7 +11154,7 @@
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A55" s="5" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="B55" s="4" t="s">
         <v>371</v>
@@ -11171,7 +11183,7 @@
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A56" s="5" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="B56" s="4" t="s">
         <v>375</v>
@@ -11192,7 +11204,7 @@
         <v>377</v>
       </c>
       <c r="H56" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I56" s="4" t="s">
         <v>379</v>
@@ -11200,7 +11212,7 @@
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A57" s="5" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="B57" s="4" t="s">
         <v>380</v>
@@ -11221,7 +11233,7 @@
         <v>382</v>
       </c>
       <c r="H57" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I57" s="4" t="s">
         <v>384</v>
@@ -11229,7 +11241,7 @@
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A58" s="5" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="B58" s="4" t="s">
         <v>385</v>
@@ -11250,7 +11262,7 @@
         <v>387</v>
       </c>
       <c r="H58" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I58" s="4" t="s">
         <v>384</v>
@@ -11258,7 +11270,7 @@
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A59" s="5" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="B59" s="4" t="s">
         <v>389</v>
@@ -11279,7 +11291,7 @@
         <v>391</v>
       </c>
       <c r="H59" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I59" s="4" t="s">
         <v>384</v>
@@ -11287,7 +11299,7 @@
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A60" s="5" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="B60" s="4" t="s">
         <v>401</v>
@@ -11308,7 +11320,7 @@
         <v>403</v>
       </c>
       <c r="H60" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I60" s="4" t="s">
         <v>405</v>
@@ -11316,7 +11328,7 @@
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A61" s="5" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="B61" s="4" t="s">
         <v>406</v>
@@ -11337,15 +11349,15 @@
         <v>408</v>
       </c>
       <c r="H61" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I61" s="4" t="s">
-        <v>410</v>
+        <v>471</v>
       </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A62" s="5" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="B62" s="4" t="s">
         <v>411</v>
@@ -11366,18 +11378,18 @@
         <v>413</v>
       </c>
       <c r="H62" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I62" s="4" t="s">
-        <v>410</v>
+        <v>471</v>
       </c>
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A63" s="5" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="B63" s="4" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="C63" s="4" t="s">
         <v>298</v>
@@ -11389,24 +11401,24 @@
         <v>55</v>
       </c>
       <c r="F63" s="4" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="G63" s="4" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="H63" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I63" s="4" t="s">
-        <v>419</v>
+        <v>472</v>
       </c>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A64" s="5" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="B64" s="4" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="C64" s="4" t="s">
         <v>298</v>
@@ -11418,24 +11430,24 @@
         <v>55</v>
       </c>
       <c r="F64" s="4" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="G64" s="4" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="H64" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I64" s="4" t="s">
-        <v>419</v>
+        <v>472</v>
       </c>
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A65" s="5" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="B65" s="4" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="C65" s="4" t="s">
         <v>212</v>
@@ -11447,24 +11459,24 @@
         <v>55</v>
       </c>
       <c r="F65" s="4" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="G65" s="4" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="H65" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I65" s="4" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A66" s="5" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="B66" s="4" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="C66" s="4" t="s">
         <v>345</v>
@@ -11476,27 +11488,27 @@
         <v>55</v>
       </c>
       <c r="F66" s="4" t="s">
+        <v>432</v>
+      </c>
+      <c r="G66" s="4" t="s">
+        <v>433</v>
+      </c>
+      <c r="H66" s="4" t="s">
+        <v>465</v>
+      </c>
+      <c r="I66" s="4" t="s">
         <v>430</v>
-      </c>
-      <c r="G66" s="4" t="s">
-        <v>431</v>
-      </c>
-      <c r="H66" s="4" t="s">
-        <v>463</v>
-      </c>
-      <c r="I66" s="4" t="s">
-        <v>428</v>
       </c>
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A67" s="5" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="B67" s="4" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="C67" s="4" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="D67" s="4" t="s">
         <v>227</v>
@@ -11505,27 +11517,27 @@
         <v>55</v>
       </c>
       <c r="F67" s="4" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="G67" s="4" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="H67" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I67" s="4" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A68" s="5" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="B68" s="4" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="C68" s="4" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="D68" s="4" t="s">
         <v>227</v>
@@ -11534,24 +11546,24 @@
         <v>55</v>
       </c>
       <c r="F68" s="4" t="s">
+        <v>442</v>
+      </c>
+      <c r="G68" s="4" t="s">
+        <v>443</v>
+      </c>
+      <c r="H68" s="4" t="s">
+        <v>465</v>
+      </c>
+      <c r="I68" s="4" t="s">
         <v>440</v>
-      </c>
-      <c r="G68" s="4" t="s">
-        <v>441</v>
-      </c>
-      <c r="H68" s="4" t="s">
-        <v>463</v>
-      </c>
-      <c r="I68" s="4" t="s">
-        <v>438</v>
       </c>
     </row>
     <row r="69" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A69" s="5" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="B69" s="4" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="C69" s="4" t="s">
         <v>361</v>
@@ -11563,27 +11575,27 @@
         <v>55</v>
       </c>
       <c r="F69" s="4" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="G69" s="4" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="H69" s="4" t="s">
         <v>365</v>
       </c>
       <c r="I69" s="4" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
     </row>
     <row r="70" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A70" s="7" t="s">
-        <v>474</v>
+        <v>478</v>
       </c>
       <c r="B70" s="4" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="C70" s="4" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="D70" s="4" t="s">
         <v>63</v>
@@ -11598,10 +11610,10 @@
         <v>63</v>
       </c>
       <c r="H70" s="4" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="I70" s="4" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Synchronize workbook conflict statuses
</commit_message>
<xml_diff>
--- a/wiring/Mazak_Wiring_Master_7i97T_7i49_7i84U_Current_Authority.xlsx
+++ b/wiring/Mazak_Wiring_Master_7i97T_7i49_7i84U_Current_Authority.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2969" uniqueCount="479">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2970" uniqueCount="479">
   <si>
     <t>Mazak VQC-20/40 Wiring Master — Current Pin Authority</t>
   </si>
@@ -1438,28 +1438,28 @@
     <t>Field Point / Load</t>
   </si>
   <si>
+    <t>Subsystem</t>
+  </si>
+  <si>
+    <t>Mesa Card</t>
+  </si>
+  <si>
+    <t>Priority</t>
+  </si>
+  <si>
+    <t>Required Action</t>
+  </si>
+  <si>
+    <t>VERIFY</t>
+  </si>
+  <si>
+    <t>BLOCKER</t>
+  </si>
+  <si>
     <t>Measure coil voltage before selecting relay contacts</t>
   </si>
   <si>
     <t>Confirm single valve versus dual coil behavior</t>
-  </si>
-  <si>
-    <t>Subsystem</t>
-  </si>
-  <si>
-    <t>Mesa Card</t>
-  </si>
-  <si>
-    <t>Priority</t>
-  </si>
-  <si>
-    <t>Required Action</t>
-  </si>
-  <si>
-    <t>VERIFY</t>
-  </si>
-  <si>
-    <t>BLOCKER</t>
   </si>
 </sst>
 </file>
@@ -6307,7 +6307,7 @@
     <pageSetUpPr fitToPage="1"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:H51"/>
+  <dimension ref="A1:H52"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0"/>
   <cols>
     <col min="1" max="3" width="16" customWidth="1"/>
@@ -6364,7 +6364,7 @@
         <v>230</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>465</v>
+        <v>40</v>
       </c>
       <c r="H2" s="4" t="s">
         <v>231</v>
@@ -6390,7 +6390,7 @@
         <v>234</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>465</v>
+        <v>40</v>
       </c>
       <c r="H3" s="4" t="s">
         <v>235</v>
@@ -6416,7 +6416,7 @@
         <v>240</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>465</v>
+        <v>40</v>
       </c>
       <c r="H4" s="4" t="s">
         <v>241</v>
@@ -6442,7 +6442,7 @@
         <v>245</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>465</v>
+        <v>40</v>
       </c>
       <c r="H5" s="4" t="s">
         <v>246</v>
@@ -6468,7 +6468,7 @@
         <v>250</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>465</v>
+        <v>40</v>
       </c>
       <c r="H6" s="4" t="s">
         <v>252</v>
@@ -6494,7 +6494,7 @@
         <v>256</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>465</v>
+        <v>40</v>
       </c>
       <c r="H7" s="4" t="s">
         <v>252</v>
@@ -6520,7 +6520,7 @@
         <v>259</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>220</v>
+        <v>40</v>
       </c>
       <c r="H8" s="4" t="s">
         <v>260</v>
@@ -6676,7 +6676,7 @@
         <v>275</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>465</v>
+        <v>40</v>
       </c>
       <c r="H14" s="4" t="s">
         <v>276</v>
@@ -6702,7 +6702,7 @@
         <v>280</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>465</v>
+        <v>40</v>
       </c>
       <c r="H15" s="4" t="s">
         <v>281</v>
@@ -6728,7 +6728,7 @@
         <v>285</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>465</v>
+        <v>40</v>
       </c>
       <c r="H16" s="4" t="s">
         <v>286</v>
@@ -6754,7 +6754,7 @@
         <v>291</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>465</v>
+        <v>40</v>
       </c>
       <c r="H17" s="4" t="s">
         <v>292</v>
@@ -6780,7 +6780,7 @@
         <v>296</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>465</v>
+        <v>40</v>
       </c>
       <c r="H18" s="4" t="s">
         <v>292</v>
@@ -6806,7 +6806,7 @@
         <v>301</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>465</v>
+        <v>40</v>
       </c>
       <c r="H19" s="4" t="s">
         <v>302</v>
@@ -6832,7 +6832,7 @@
         <v>306</v>
       </c>
       <c r="G20" s="4" t="s">
-        <v>465</v>
+        <v>40</v>
       </c>
       <c r="H20" s="4" t="s">
         <v>307</v>
@@ -6858,7 +6858,7 @@
         <v>312</v>
       </c>
       <c r="G21" s="4" t="s">
-        <v>465</v>
+        <v>40</v>
       </c>
       <c r="H21" s="4" t="s">
         <v>252</v>
@@ -6884,7 +6884,7 @@
         <v>316</v>
       </c>
       <c r="G22" s="4" t="s">
-        <v>465</v>
+        <v>40</v>
       </c>
       <c r="H22" s="4" t="s">
         <v>252</v>
@@ -6910,7 +6910,7 @@
         <v>321</v>
       </c>
       <c r="G23" s="4" t="s">
-        <v>465</v>
+        <v>40</v>
       </c>
       <c r="H23" s="4" t="s">
         <v>322</v>
@@ -6936,7 +6936,7 @@
         <v>326</v>
       </c>
       <c r="G24" s="4" t="s">
-        <v>465</v>
+        <v>40</v>
       </c>
       <c r="H24" s="4" t="s">
         <v>322</v>
@@ -6962,7 +6962,7 @@
         <v>330</v>
       </c>
       <c r="G25" s="4" t="s">
-        <v>465</v>
+        <v>40</v>
       </c>
       <c r="H25" s="4" t="s">
         <v>322</v>
@@ -6988,7 +6988,7 @@
         <v>334</v>
       </c>
       <c r="G26" s="4" t="s">
-        <v>465</v>
+        <v>40</v>
       </c>
       <c r="H26" s="4" t="s">
         <v>322</v>
@@ -7014,7 +7014,7 @@
         <v>338</v>
       </c>
       <c r="G27" s="4" t="s">
-        <v>465</v>
+        <v>40</v>
       </c>
       <c r="H27" s="4" t="s">
         <v>322</v>
@@ -7040,7 +7040,7 @@
         <v>342</v>
       </c>
       <c r="G28" s="4" t="s">
-        <v>465</v>
+        <v>40</v>
       </c>
       <c r="H28" s="4" t="s">
         <v>343</v>
@@ -7066,7 +7066,7 @@
         <v>348</v>
       </c>
       <c r="G29" s="4" t="s">
-        <v>465</v>
+        <v>40</v>
       </c>
       <c r="H29" s="4" t="s">
         <v>349</v>
@@ -7092,7 +7092,7 @@
         <v>353</v>
       </c>
       <c r="G30" s="4" t="s">
-        <v>465</v>
+        <v>40</v>
       </c>
       <c r="H30" s="4" t="s">
         <v>349</v>
@@ -7118,7 +7118,7 @@
         <v>358</v>
       </c>
       <c r="G31" s="4" t="s">
-        <v>465</v>
+        <v>40</v>
       </c>
       <c r="H31" s="4" t="s">
         <v>359</v>
@@ -7144,7 +7144,7 @@
         <v>364</v>
       </c>
       <c r="G32" s="4" t="s">
-        <v>365</v>
+        <v>40</v>
       </c>
       <c r="H32" s="4" t="s">
         <v>366</v>
@@ -7222,7 +7222,7 @@
         <v>378</v>
       </c>
       <c r="G35" s="4" t="s">
-        <v>465</v>
+        <v>365</v>
       </c>
       <c r="H35" s="4" t="s">
         <v>379</v>
@@ -7248,7 +7248,7 @@
         <v>383</v>
       </c>
       <c r="G36" s="4" t="s">
-        <v>465</v>
+        <v>40</v>
       </c>
       <c r="H36" s="4" t="s">
         <v>384</v>
@@ -7274,7 +7274,7 @@
         <v>388</v>
       </c>
       <c r="G37" s="4" t="s">
-        <v>465</v>
+        <v>40</v>
       </c>
       <c r="H37" s="4" t="s">
         <v>384</v>
@@ -7300,7 +7300,7 @@
         <v>392</v>
       </c>
       <c r="G38" s="4" t="s">
-        <v>465</v>
+        <v>40</v>
       </c>
       <c r="H38" s="4" t="s">
         <v>384</v>
@@ -7326,7 +7326,7 @@
         <v>395</v>
       </c>
       <c r="G39" s="4" t="s">
-        <v>220</v>
+        <v>40</v>
       </c>
       <c r="H39" s="4" t="s">
         <v>396</v>
@@ -7404,7 +7404,7 @@
         <v>404</v>
       </c>
       <c r="G42" s="4" t="s">
-        <v>465</v>
+        <v>220</v>
       </c>
       <c r="H42" s="4" t="s">
         <v>405</v>
@@ -7430,10 +7430,10 @@
         <v>409</v>
       </c>
       <c r="G43" s="4" t="s">
-        <v>465</v>
+        <v>40</v>
       </c>
       <c r="H43" s="4" t="s">
-        <v>471</v>
+        <v>410</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.25">
@@ -7456,10 +7456,10 @@
         <v>414</v>
       </c>
       <c r="G44" s="4" t="s">
-        <v>465</v>
+        <v>103</v>
       </c>
       <c r="H44" s="4" t="s">
-        <v>471</v>
+        <v>415</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.25">
@@ -7482,10 +7482,10 @@
         <v>419</v>
       </c>
       <c r="G45" s="4" t="s">
-        <v>465</v>
+        <v>103</v>
       </c>
       <c r="H45" s="4" t="s">
-        <v>472</v>
+        <v>420</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.25">
@@ -7508,10 +7508,10 @@
         <v>424</v>
       </c>
       <c r="G46" s="4" t="s">
-        <v>465</v>
+        <v>103</v>
       </c>
       <c r="H46" s="4" t="s">
-        <v>472</v>
+        <v>425</v>
       </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.25">
@@ -7534,7 +7534,7 @@
         <v>429</v>
       </c>
       <c r="G47" s="4" t="s">
-        <v>465</v>
+        <v>40</v>
       </c>
       <c r="H47" s="4" t="s">
         <v>430</v>
@@ -7560,7 +7560,7 @@
         <v>434</v>
       </c>
       <c r="G48" s="4" t="s">
-        <v>465</v>
+        <v>40</v>
       </c>
       <c r="H48" s="4" t="s">
         <v>430</v>
@@ -7586,7 +7586,7 @@
         <v>439</v>
       </c>
       <c r="G49" s="4" t="s">
-        <v>465</v>
+        <v>40</v>
       </c>
       <c r="H49" s="4" t="s">
         <v>440</v>
@@ -7612,7 +7612,7 @@
         <v>444</v>
       </c>
       <c r="G50" s="4" t="s">
-        <v>465</v>
+        <v>40</v>
       </c>
       <c r="H50" s="4" t="s">
         <v>440</v>
@@ -7638,10 +7638,15 @@
         <v>448</v>
       </c>
       <c r="G51" s="4" t="s">
-        <v>365</v>
+        <v>40</v>
       </c>
       <c r="H51" s="4" t="s">
         <v>450</v>
+      </c>
+    </row>
+    <row r="52" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G52" t="s">
+        <v>365</v>
       </c>
     </row>
   </sheetData>
@@ -7680,13 +7685,13 @@
         <v>459</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
       <c r="D1" s="3" t="s">
         <v>462</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="F1" s="3" t="s">
         <v>457</v>
@@ -9588,16 +9593,16 @@
   <sheetData>
     <row r="1" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>459</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="E1" s="3" t="s">
         <v>457</v>
@@ -9612,12 +9617,12 @@
         <v>463</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>32</v>
@@ -9646,7 +9651,7 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>43</v>
@@ -9675,7 +9680,7 @@
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>47</v>
@@ -9704,7 +9709,7 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B5" s="4" t="s">
         <v>51</v>
@@ -9733,7 +9738,7 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>68</v>
@@ -9762,7 +9767,7 @@
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B7" s="4" t="s">
         <v>75</v>
@@ -9791,7 +9796,7 @@
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B8" s="4" t="s">
         <v>81</v>
@@ -9820,7 +9825,7 @@
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B9" s="4" t="s">
         <v>85</v>
@@ -9849,7 +9854,7 @@
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B10" s="4" t="s">
         <v>90</v>
@@ -9878,7 +9883,7 @@
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B11" s="4" t="s">
         <v>94</v>
@@ -9907,7 +9912,7 @@
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
-        <v>478</v>
+        <v>476</v>
       </c>
       <c r="B12" s="4" t="s">
         <v>99</v>
@@ -9936,7 +9941,7 @@
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B13" s="4" t="s">
         <v>105</v>
@@ -9965,7 +9970,7 @@
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B14" s="4" t="s">
         <v>143</v>
@@ -9994,7 +9999,7 @@
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B15" s="4" t="s">
         <v>152</v>
@@ -10023,7 +10028,7 @@
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B16" s="4" t="s">
         <v>156</v>
@@ -10052,7 +10057,7 @@
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B17" s="4" t="s">
         <v>160</v>
@@ -10081,7 +10086,7 @@
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B18" s="4" t="s">
         <v>164</v>
@@ -10110,7 +10115,7 @@
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B19" s="4" t="s">
         <v>168</v>
@@ -10139,7 +10144,7 @@
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B20" s="4" t="s">
         <v>172</v>
@@ -10168,7 +10173,7 @@
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B21" s="4" t="s">
         <v>176</v>
@@ -10197,7 +10202,7 @@
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B22" s="4" t="s">
         <v>180</v>
@@ -10226,7 +10231,7 @@
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B23" s="4" t="s">
         <v>184</v>
@@ -10255,7 +10260,7 @@
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B24" s="4" t="s">
         <v>190</v>
@@ -10284,7 +10289,7 @@
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B25" s="4" t="s">
         <v>196</v>
@@ -10313,7 +10318,7 @@
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B26" s="4" t="s">
         <v>200</v>
@@ -10342,7 +10347,7 @@
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" s="5" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B27" s="4" t="s">
         <v>207</v>
@@ -10371,7 +10376,7 @@
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" s="5" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B28" s="4" t="s">
         <v>211</v>
@@ -10400,7 +10405,7 @@
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" s="5" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B29" s="4" t="s">
         <v>226</v>
@@ -10429,7 +10434,7 @@
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" s="5" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B30" s="4" t="s">
         <v>232</v>
@@ -10458,7 +10463,7 @@
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" s="5" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B31" s="4" t="s">
         <v>236</v>
@@ -10487,7 +10492,7 @@
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" s="5" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B32" s="4" t="s">
         <v>242</v>
@@ -10516,7 +10521,7 @@
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" s="5" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B33" s="4" t="s">
         <v>247</v>
@@ -10545,7 +10550,7 @@
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" s="5" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B34" s="4" t="s">
         <v>253</v>
@@ -10574,7 +10579,7 @@
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" s="5" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B35" s="4" t="s">
         <v>271</v>
@@ -10603,7 +10608,7 @@
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" s="5" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B36" s="4" t="s">
         <v>277</v>
@@ -10632,7 +10637,7 @@
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" s="5" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B37" s="4" t="s">
         <v>282</v>
@@ -10661,7 +10666,7 @@
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" s="5" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B38" s="4" t="s">
         <v>287</v>
@@ -10690,7 +10695,7 @@
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" s="5" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B39" s="4" t="s">
         <v>293</v>
@@ -10719,7 +10724,7 @@
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" s="5" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B40" s="4" t="s">
         <v>297</v>
@@ -10748,7 +10753,7 @@
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" s="5" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B41" s="4" t="s">
         <v>303</v>
@@ -10777,7 +10782,7 @@
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" s="5" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B42" s="4" t="s">
         <v>308</v>
@@ -10806,7 +10811,7 @@
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" s="5" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B43" s="4" t="s">
         <v>313</v>
@@ -10835,7 +10840,7 @@
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" s="5" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B44" s="4" t="s">
         <v>317</v>
@@ -10864,7 +10869,7 @@
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" s="5" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B45" s="4" t="s">
         <v>323</v>
@@ -10893,7 +10898,7 @@
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46" s="5" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B46" s="4" t="s">
         <v>327</v>
@@ -10922,7 +10927,7 @@
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47" s="5" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B47" s="4" t="s">
         <v>331</v>
@@ -10951,7 +10956,7 @@
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" s="5" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B48" s="4" t="s">
         <v>335</v>
@@ -10980,7 +10985,7 @@
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A49" s="5" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B49" s="4" t="s">
         <v>339</v>
@@ -11009,7 +11014,7 @@
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A50" s="5" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B50" s="4" t="s">
         <v>344</v>
@@ -11038,7 +11043,7 @@
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A51" s="5" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B51" s="4" t="s">
         <v>350</v>
@@ -11067,7 +11072,7 @@
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A52" s="5" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B52" s="4" t="s">
         <v>354</v>
@@ -11096,7 +11101,7 @@
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A53" s="5" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B53" s="4" t="s">
         <v>360</v>
@@ -11125,7 +11130,7 @@
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A54" s="5" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B54" s="4" t="s">
         <v>367</v>
@@ -11154,7 +11159,7 @@
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A55" s="5" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B55" s="4" t="s">
         <v>371</v>
@@ -11183,7 +11188,7 @@
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A56" s="5" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B56" s="4" t="s">
         <v>375</v>
@@ -11212,7 +11217,7 @@
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A57" s="5" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B57" s="4" t="s">
         <v>380</v>
@@ -11241,7 +11246,7 @@
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A58" s="5" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B58" s="4" t="s">
         <v>385</v>
@@ -11270,7 +11275,7 @@
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A59" s="5" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B59" s="4" t="s">
         <v>389</v>
@@ -11299,7 +11304,7 @@
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A60" s="5" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B60" s="4" t="s">
         <v>401</v>
@@ -11328,7 +11333,7 @@
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A61" s="5" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B61" s="4" t="s">
         <v>406</v>
@@ -11352,12 +11357,12 @@
         <v>465</v>
       </c>
       <c r="I61" s="4" t="s">
-        <v>471</v>
+        <v>477</v>
       </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A62" s="5" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B62" s="4" t="s">
         <v>411</v>
@@ -11381,12 +11386,12 @@
         <v>465</v>
       </c>
       <c r="I62" s="4" t="s">
-        <v>471</v>
+        <v>477</v>
       </c>
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A63" s="5" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B63" s="4" t="s">
         <v>416</v>
@@ -11410,12 +11415,12 @@
         <v>465</v>
       </c>
       <c r="I63" s="4" t="s">
-        <v>472</v>
+        <v>478</v>
       </c>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A64" s="5" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B64" s="4" t="s">
         <v>421</v>
@@ -11439,12 +11444,12 @@
         <v>465</v>
       </c>
       <c r="I64" s="4" t="s">
-        <v>472</v>
+        <v>478</v>
       </c>
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A65" s="5" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B65" s="4" t="s">
         <v>426</v>
@@ -11473,7 +11478,7 @@
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A66" s="5" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B66" s="4" t="s">
         <v>431</v>
@@ -11502,7 +11507,7 @@
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A67" s="5" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B67" s="4" t="s">
         <v>435</v>
@@ -11531,7 +11536,7 @@
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A68" s="5" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B68" s="4" t="s">
         <v>441</v>
@@ -11560,7 +11565,7 @@
     </row>
     <row r="69" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A69" s="5" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B69" s="4" t="s">
         <v>445</v>
@@ -11589,7 +11594,7 @@
     </row>
     <row r="70" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A70" s="7" t="s">
-        <v>478</v>
+        <v>476</v>
       </c>
       <c r="B70" s="4" t="s">
         <v>451</v>

</xml_diff>